<commit_message>
fix: match original Excel layout and localize form validation and sources (v1.0.1)
</commit_message>
<xml_diff>
--- a/templates/成品日检表模板.xlsx
+++ b/templates/成品日检表模板.xlsx
@@ -701,7 +701,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -838,6 +838,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
@@ -969,74 +972,261 @@
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>不良项目出现批次</a:t>
+              <a:t>返工批次</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <layout/>
+      <overlay val="0"/>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.0230039286793593"/>
+          <y val="0.104109589041096"/>
+          <w val="0.95871123155676"/>
+          <h val="0.432146118721461"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
             <a:ln>
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
-              <f>'数据分析表'!$A$4:$A$27</f>
-            </numRef>
+            <strRef>
+              <f>数据分析表!$E$4:$E$11</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'数据分析表'!$B$4:$B$27</f>
+              <f>数据分析表!$F$4:$F$11</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="219"/>
+        <overlap val="-27"/>
+        <axId val="616496748"/>
+        <axId val="27574989"/>
       </barChart>
       <catAx>
-        <axId val="10"/>
+        <axId val="616496748"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="27574989"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="100"/>
+        <axId val="27574989"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="10"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="616496748"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -1046,74 +1236,249 @@
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>组别返工批次</a:t>
+              <a:t>抽检状况统计表</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <layout/>
+      <overlay val="0"/>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </title>
     <plotArea>
+      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
             <a:ln>
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
-              <f>'数据分析表'!$E$4:$E$11</f>
-            </numRef>
+            <strRef>
+              <f>数据分析表!$H$3:$K$3</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'数据分析表'!$F$4:$F$11</f>
+              <f>数据分析表!$H$4:$K$4</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="219"/>
+        <overlap val="-27"/>
+        <axId val="731071656"/>
+        <axId val="503185410"/>
       </barChart>
       <catAx>
-        <axId val="10"/>
+        <axId val="731071656"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="503185410"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="100"/>
+        <axId val="503185410"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="10"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="731071656"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -1123,74 +1488,249 @@
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>检验数量</a:t>
+              <a:t>不良项汇总</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <layout/>
+      <overlay val="0"/>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </title>
     <plotArea>
+      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
             <a:ln>
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
-              <f>'数据分析表'!$H$4</f>
-            </numRef>
+            <strRef>
+              <f>数据分析表!$A$4:$A$27</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'数据分析表'!$H$4</f>
+              <f>数据分析表!$B$4:$B$27</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="219"/>
+        <overlap val="-27"/>
+        <axId val="135544323"/>
+        <axId val="648306811"/>
       </barChart>
       <catAx>
-        <axId val="10"/>
+        <axId val="135544323"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="648306811"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="100"/>
+        <axId val="648306811"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="10"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="135544323"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -1200,74 +1740,249 @@
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>不良项目出现批次</a:t>
+              <a:t>抽检状况统计表</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <layout/>
+      <overlay val="0"/>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </title>
     <plotArea>
+      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
             <a:ln>
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
-              <f>'数据分析表'!$A$34:$A$57</f>
-            </numRef>
+            <strRef>
+              <f>数据分析表!$H$33:$K$33</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'数据分析表'!$B$34:$B$57</f>
+              <f>数据分析表!$H$34:$K$34</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="219"/>
+        <overlap val="-27"/>
+        <axId val="731071656"/>
+        <axId val="503185410"/>
       </barChart>
       <catAx>
-        <axId val="10"/>
+        <axId val="731071656"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="503185410"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="100"/>
+        <axId val="503185410"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="10"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="731071656"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -1277,74 +1992,313 @@
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>组别返工批次</a:t>
+              <a:t>每周抽检不良项目统计</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <layout/>
+      <overlay val="0"/>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </title>
     <plotArea>
+      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
             <a:ln>
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
-              <f>'数据分析表'!$E$34:$E$41</f>
-            </numRef>
+            <strRef>
+              <f>数据分析表!$A$34:$A$57</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'数据分析表'!$F$34:$F$41</f>
+              <f>数据分析表!$B$34:$B$57</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="General"/>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
+          <cat>
+            <strRef>
+              <f>数据分析表!$A$34:$A$57</f>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>数据分析表!$C$34:$C$57</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="219"/>
+        <overlap val="-27"/>
+        <axId val="965444067"/>
+        <axId val="789959763"/>
       </barChart>
       <catAx>
-        <axId val="10"/>
+        <axId val="965444067"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="789959763"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="100"/>
+        <axId val="789959763"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="10"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="965444067"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -1354,87 +2308,267 @@
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
           <a:p>
-            <a:pPr>
-              <a:defRPr/>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>检验数量</a:t>
+              <a:t>每周返工批次统计</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
+      <layout/>
+      <overlay val="0"/>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </title>
     <plotArea>
+      <layout/>
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
             <a:ln>
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="outEnd"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
           <cat>
-            <numRef>
-              <f>'数据分析表'!$H$34</f>
-            </numRef>
+            <strRef>
+              <f>数据分析表!$E$34:$E$41</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'数据分析表'!$H$34</f>
+              <f>数据分析表!$F$34:$F$41</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="219"/>
+        <overlap val="-27"/>
+        <axId val="278395373"/>
+        <axId val="922167448"/>
       </barChart>
       <catAx>
-        <axId val="10"/>
+        <axId val="278395373"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <delete val="0"/>
+        <axPos val="b"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="100"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="922167448"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
         <lblOffset val="100"/>
+        <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="100"/>
+        <axId val="922167448"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="General" sourceLinked="1"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
-        <crossAx val="10"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
+        <crossAx val="278395373"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
       </valAx>
     </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
+  <twoCellAnchor>
     <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>62</row>
-      <rowOff>0</rowOff>
+      <col>4</col>
+      <colOff>3175</colOff>
+      <row>12</row>
+      <rowOff>69850</rowOff>
     </from>
-    <ext cx="4680000" cy="2880000"/>
+    <to>
+      <col>11</col>
+      <colOff>41275</colOff>
+      <row>17</row>
+      <rowOff>117475</rowOff>
+    </to>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1448,15 +2582,20 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
+  </twoCellAnchor>
+  <twoCellAnchor>
     <from>
-      <col>5</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>62</row>
-      <rowOff>0</rowOff>
+      <row>4</row>
+      <rowOff>60325</rowOff>
     </from>
-    <ext cx="4680000" cy="2880000"/>
+    <to>
+      <col>11</col>
+      <colOff>22225</colOff>
+      <row>12</row>
+      <rowOff>3175</rowOff>
+    </to>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1470,15 +2609,20 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
+  </twoCellAnchor>
+  <twoCellAnchor>
     <from>
-      <col>10</col>
-      <colOff>0</colOff>
-      <row>62</row>
-      <rowOff>0</rowOff>
+      <col>4</col>
+      <colOff>9525</colOff>
+      <row>17</row>
+      <rowOff>155575</rowOff>
     </from>
-    <ext cx="4680000" cy="2880000"/>
+    <to>
+      <col>11</col>
+      <colOff>57150</colOff>
+      <row>27</row>
+      <rowOff>212725</rowOff>
+    </to>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1492,15 +2636,20 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
+  </twoCellAnchor>
+  <twoCellAnchor>
     <from>
-      <col>0</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>80</row>
-      <rowOff>0</rowOff>
+      <row>34</row>
+      <rowOff>60325</rowOff>
     </from>
-    <ext cx="4680000" cy="2880000"/>
+    <to>
+      <col>11</col>
+      <colOff>22225</colOff>
+      <row>41</row>
+      <rowOff>222250</rowOff>
+    </to>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1514,15 +2663,20 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
+  </twoCellAnchor>
+  <twoCellAnchor>
     <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>80</row>
-      <rowOff>0</rowOff>
+      <col>3</col>
+      <colOff>692150</colOff>
+      <row>49</row>
+      <rowOff>384175</rowOff>
     </from>
-    <ext cx="4680000" cy="2880000"/>
+    <to>
+      <col>11</col>
+      <colOff>2540</colOff>
+      <row>57</row>
+      <rowOff>231775</rowOff>
+    </to>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="5" name="Chart 5"/>
@@ -1536,15 +2690,20 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
+  </twoCellAnchor>
+  <twoCellAnchor>
     <from>
-      <col>10</col>
-      <colOff>0</colOff>
-      <row>80</row>
-      <rowOff>0</rowOff>
+      <col>3</col>
+      <colOff>692150</colOff>
+      <row>42</row>
+      <rowOff>47625</rowOff>
     </from>
-    <ext cx="4680000" cy="2880000"/>
+    <to>
+      <col>11</col>
+      <colOff>12065</colOff>
+      <row>49</row>
+      <rowOff>333375</rowOff>
+    </to>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="6" name="Chart 6"/>
@@ -1558,7 +2717,7 @@
       </a:graphic>
     </graphicFrame>
     <clientData/>
-  </oneCellAnchor>
+  </twoCellAnchor>
 </wsDr>
 </file>
 
@@ -1901,299 +3060,6 @@
       <c r="I2" s="42" t="n"/>
       <c r="J2" s="25" t="n"/>
     </row>
-    <row r="3" ht="34.45" customHeight="1" s="45"/>
-    <row r="4" ht="33.95" customHeight="1" s="45"/>
-    <row r="5" ht="36.9" customHeight="1" s="45"/>
-    <row r="6" ht="33.95" customHeight="1" s="45"/>
-    <row r="7" ht="33.95" customHeight="1" s="45"/>
-    <row r="8" ht="36.9" customHeight="1" s="45"/>
-    <row r="9" ht="36.9" customHeight="1" s="45"/>
-    <row r="10" ht="36.2" customHeight="1" s="45"/>
-    <row r="11" ht="36.2" customHeight="1" s="45"/>
-    <row r="12" ht="36.9" customHeight="1" s="45"/>
-    <row r="13" ht="36.9" customHeight="1" s="45"/>
-    <row r="14" ht="34.4" customHeight="1" s="45"/>
-    <row r="15" ht="34.4" customHeight="1" s="45"/>
-    <row r="16" ht="34.4" customHeight="1" s="45"/>
-    <row r="17" ht="36.2" customHeight="1" s="45"/>
-    <row r="18" ht="36.2" customHeight="1" s="45"/>
-    <row r="19" ht="36.2" customHeight="1" s="45"/>
-    <row r="20" ht="36.2" customHeight="1" s="45"/>
-    <row r="21" ht="36.9" customHeight="1" s="45"/>
-    <row r="22" ht="36.9" customHeight="1" s="45"/>
-    <row r="23" ht="36.9" customHeight="1" s="45"/>
-    <row r="24" ht="36.9" customHeight="1" s="45"/>
-    <row r="25" ht="34.4" customHeight="1" s="45"/>
-    <row r="26" ht="34.4" customHeight="1" s="45"/>
-    <row r="27" ht="34.4" customHeight="1" s="45"/>
-    <row r="28" ht="33.95" customHeight="1" s="45"/>
-    <row r="29" ht="33.95" customHeight="1" s="45"/>
-    <row r="30" ht="33.95" customHeight="1" s="45"/>
-    <row r="31" ht="36.2" customHeight="1" s="45"/>
-    <row r="32" ht="36.2" customHeight="1" s="45"/>
-    <row r="33" ht="36.2" customHeight="1" s="45"/>
-    <row r="34" ht="36.2" customHeight="1" s="45"/>
-    <row r="35" ht="36.2" customHeight="1" s="45"/>
-    <row r="36" ht="36.2" customHeight="1" s="45"/>
-    <row r="37" ht="36.2" customHeight="1" s="45"/>
-    <row r="38" ht="36.2" customHeight="1" s="45"/>
-    <row r="39" ht="34.4" customHeight="1" s="45"/>
-    <row r="40" ht="34.4" customHeight="1" s="45"/>
-    <row r="41" ht="34.4" customHeight="1" s="45"/>
-    <row r="42" ht="34.4" customHeight="1" s="45"/>
-    <row r="43" ht="36.2" customHeight="1" s="45"/>
-    <row r="44" ht="36.2" customHeight="1" s="45"/>
-    <row r="45" ht="36.9" customHeight="1" s="45"/>
-    <row r="46" ht="36.9" customHeight="1" s="45"/>
-    <row r="47" ht="34.4" customHeight="1" s="45"/>
-    <row r="48" ht="36.9" customHeight="1" s="45"/>
-    <row r="49" ht="34.4" customHeight="1" s="45"/>
-    <row r="50" ht="34.4" customHeight="1" s="45"/>
-    <row r="51" ht="36.9" customHeight="1" s="45"/>
-    <row r="52" ht="36.2" customHeight="1" s="45"/>
-    <row r="53" ht="36.2" customHeight="1" s="45"/>
-    <row r="54" ht="36.2" customHeight="1" s="45"/>
-    <row r="55" ht="34.4" customHeight="1" s="45"/>
-    <row r="56" ht="34.4" customHeight="1" s="45"/>
-    <row r="57" ht="34.4" customHeight="1" s="45"/>
-    <row r="58" ht="36.9" customHeight="1" s="45"/>
-    <row r="59" ht="36.9" customHeight="1" s="45"/>
-    <row r="60" ht="36.2" customHeight="1" s="45"/>
-    <row r="61" ht="36.2" customHeight="1" s="45"/>
-    <row r="62" ht="34.4" customHeight="1" s="45"/>
-    <row r="63" ht="34.4" customHeight="1" s="45"/>
-    <row r="64" ht="34.4" customHeight="1" s="45"/>
-    <row r="65" ht="34.4" customHeight="1" s="45"/>
-    <row r="66" ht="36.9" customHeight="1" s="45"/>
-    <row r="67" ht="34.4" customHeight="1" s="45"/>
-    <row r="68" ht="36.9" customHeight="1" s="45"/>
-    <row r="69" ht="34.4" customHeight="1" s="45"/>
-    <row r="70" ht="36.9" customHeight="1" s="45"/>
-    <row r="71" ht="34.4" customHeight="1" s="45"/>
-    <row r="72" ht="34.4" customHeight="1" s="45"/>
-    <row r="73" ht="34.4" customHeight="1" s="45"/>
-    <row r="74" ht="36.9" customHeight="1" s="45"/>
-    <row r="75" ht="36.9" customHeight="1" s="45"/>
-    <row r="76" ht="34.4" customHeight="1" s="45"/>
-    <row r="77" ht="34.4" customHeight="1" s="45"/>
-    <row r="78" ht="34.4" customHeight="1" s="45"/>
-    <row r="79" ht="36.9" customHeight="1" s="45"/>
-    <row r="80" ht="36.9" customHeight="1" s="45"/>
-    <row r="81" ht="36.9" customHeight="1" s="45"/>
-    <row r="82" ht="33.95" customHeight="1" s="45"/>
-    <row r="83" ht="33.95" customHeight="1" s="45"/>
-    <row r="84" ht="33.95" customHeight="1" s="45"/>
-    <row r="85" ht="33.95" customHeight="1" s="45"/>
-    <row r="86" ht="36.2" customHeight="1" s="45"/>
-    <row r="87" ht="36.2" customHeight="1" s="45"/>
-    <row r="88" ht="36.2" customHeight="1" s="45"/>
-    <row r="89" ht="36.2" customHeight="1" s="45"/>
-    <row r="90" ht="36.2" customHeight="1" s="45"/>
-    <row r="91" ht="36.2" customHeight="1" s="45"/>
-    <row r="92" ht="36.2" customHeight="1" s="45"/>
-    <row r="93" ht="36.2" customHeight="1" s="45"/>
-    <row r="94" ht="36.2" customHeight="1" s="45"/>
-    <row r="95" ht="36.2" customHeight="1" s="45"/>
-    <row r="96" ht="36.2" customHeight="1" s="45"/>
-    <row r="97" ht="36.9" customHeight="1" s="45"/>
-    <row r="98" ht="36.9" customHeight="1" s="45"/>
-    <row r="99" ht="33.95" customHeight="1" s="45"/>
-    <row r="100" ht="33.95" customHeight="1" s="45"/>
-    <row r="101" ht="33.95" customHeight="1" s="45"/>
-    <row r="102" ht="36.9" customHeight="1" s="45"/>
-    <row r="103" ht="33.95" customHeight="1" s="45"/>
-    <row r="104" ht="33.95" customHeight="1" s="45"/>
-    <row r="105" ht="33.95" customHeight="1" s="45"/>
-    <row r="106" ht="33.95" customHeight="1" s="45"/>
-    <row r="107" ht="36.2" customHeight="1" s="45"/>
-    <row r="108" ht="36.2" customHeight="1" s="45"/>
-    <row r="109" ht="36.2" customHeight="1" s="45"/>
-    <row r="110" ht="36.2" customHeight="1" s="45"/>
-    <row r="111" ht="33.95" customHeight="1" s="45"/>
-    <row r="112" ht="33.95" customHeight="1" s="45"/>
-    <row r="113" ht="33.95" customHeight="1" s="45"/>
-    <row r="114" ht="36.9" customHeight="1" s="45"/>
-    <row r="115" ht="36.9" customHeight="1" s="45"/>
-    <row r="116" ht="36.2" customHeight="1" s="45"/>
-    <row r="117" ht="36.2" customHeight="1" s="45"/>
-    <row r="118" ht="33.95" customHeight="1" s="45"/>
-    <row r="119" ht="33.95" customHeight="1" s="45"/>
-    <row r="120" ht="33.95" customHeight="1" s="45"/>
-    <row r="121" ht="33.95" customHeight="1" s="45"/>
-    <row r="122" ht="36.9" customHeight="1" s="45"/>
-    <row r="123" ht="36.9" customHeight="1" s="45"/>
-    <row r="124" ht="36.2" customHeight="1" s="45"/>
-    <row r="125" ht="36.2" customHeight="1" s="45"/>
-    <row r="126" ht="33.95" customHeight="1" s="45"/>
-    <row r="127" ht="33.95" customHeight="1" s="45"/>
-    <row r="128" ht="33.95" customHeight="1" s="45"/>
-    <row r="129" ht="33.95" customHeight="1" s="45"/>
-    <row r="130" ht="36.9" customHeight="1" s="45"/>
-    <row r="131" ht="36.9" customHeight="1" s="45"/>
-    <row r="132" ht="36.2" customHeight="1" s="45"/>
-    <row r="133" ht="36.2" customHeight="1" s="45"/>
-    <row r="134" ht="33.95" customHeight="1" s="45"/>
-    <row r="135" ht="33.95" customHeight="1" s="45"/>
-    <row r="136" ht="33.95" customHeight="1" s="45"/>
-    <row r="137" ht="36.9" customHeight="1" s="45"/>
-    <row r="138" ht="36.9" customHeight="1" s="45"/>
-    <row r="139" ht="33.95" customHeight="1" s="45"/>
-    <row r="140" ht="33.95" customHeight="1" s="45"/>
-    <row r="141" ht="33.95" customHeight="1" s="45"/>
-    <row r="142" ht="33.95" customHeight="1" s="45"/>
-    <row r="143" ht="36.2" customHeight="1" s="45"/>
-    <row r="144" ht="36.2" customHeight="1" s="45"/>
-    <row r="145" ht="36.2" customHeight="1" s="45"/>
-    <row r="146" ht="33.95" customHeight="1" s="45"/>
-    <row r="147" ht="33.95" customHeight="1" s="45"/>
-    <row r="148" ht="33.95" customHeight="1" s="45"/>
-    <row r="149" ht="36.9" customHeight="1" s="45"/>
-    <row r="150" ht="36.9" customHeight="1" s="45"/>
-    <row r="151" ht="36.9" customHeight="1" s="45"/>
-    <row r="152" ht="36.9" customHeight="1" s="45"/>
-    <row r="153" ht="33.95" customHeight="1" s="45"/>
-    <row r="154" ht="33.95" customHeight="1" s="45"/>
-    <row r="155" ht="33.95" customHeight="1" s="45"/>
-    <row r="156" ht="33.95" customHeight="1" s="45"/>
-    <row r="157" ht="33.95" customHeight="1" s="45"/>
-    <row r="158" ht="33.95" customHeight="1" s="45"/>
-    <row r="159" ht="33.95" customHeight="1" s="45"/>
-    <row r="160" ht="33.95" customHeight="1" s="45"/>
-    <row r="161" ht="36.9" customHeight="1" s="45"/>
-    <row r="162" ht="36.9" customHeight="1" s="45"/>
-    <row r="163" ht="33.95" customHeight="1" s="45"/>
-    <row r="164" ht="33.95" customHeight="1" s="45"/>
-    <row r="165" ht="33.95" customHeight="1" s="45"/>
-    <row r="166" ht="36.9" customHeight="1" s="45"/>
-    <row r="167" ht="36.9" customHeight="1" s="45"/>
-    <row r="168" ht="36.9" customHeight="1" s="45"/>
-    <row r="169" ht="36.9" customHeight="1" s="45"/>
-    <row r="170" ht="33.95" customHeight="1" s="45"/>
-    <row r="171" ht="33.95" customHeight="1" s="45"/>
-    <row r="172" ht="36.9" customHeight="1" s="45"/>
-    <row r="173" ht="33.95" customHeight="1" s="45"/>
-    <row r="174" ht="33.95" customHeight="1" s="45"/>
-    <row r="175" ht="33.95" customHeight="1" s="45"/>
-    <row r="176" ht="36.2" customHeight="1" s="45"/>
-    <row r="177" ht="36.2" customHeight="1" s="45"/>
-    <row r="178" ht="36.2" customHeight="1" s="45"/>
-    <row r="179" ht="36.2" customHeight="1" s="45"/>
-    <row r="180" ht="33.95" customHeight="1" s="45"/>
-    <row r="181" ht="33.95" customHeight="1" s="45"/>
-    <row r="182" ht="33.95" customHeight="1" s="45"/>
-    <row r="183" ht="36.9" customHeight="1" s="45"/>
-    <row r="184" ht="36.9" customHeight="1" s="45"/>
-    <row r="185" ht="36.2" customHeight="1" s="45"/>
-    <row r="186" ht="36.2" customHeight="1" s="45"/>
-    <row r="187" ht="36.2" customHeight="1" s="45"/>
-    <row r="188" ht="36.2" customHeight="1" s="45"/>
-    <row r="189" ht="33.95" customHeight="1" s="45"/>
-    <row r="190" ht="33.95" customHeight="1" s="45"/>
-    <row r="191" ht="33.95" customHeight="1" s="45"/>
-    <row r="192" ht="36.9" customHeight="1" s="45"/>
-    <row r="193" ht="36.9" customHeight="1" s="45"/>
-    <row r="194" ht="33.95" customHeight="1" s="45"/>
-    <row r="195" ht="33.95" customHeight="1" s="45"/>
-    <row r="196" ht="33.95" customHeight="1" s="45"/>
-    <row r="197" ht="33.95" customHeight="1" s="45"/>
-    <row r="198" ht="36.9" customHeight="1" s="45"/>
-    <row r="199" ht="36.9" customHeight="1" s="45"/>
-    <row r="200" ht="33.95" customHeight="1" s="45"/>
-    <row r="201" ht="33.95" customHeight="1" s="45"/>
-    <row r="202" ht="33.95" customHeight="1" s="45"/>
-    <row r="203" ht="33.95" customHeight="1" s="45"/>
-    <row r="204" ht="36.2" customHeight="1" s="45"/>
-    <row r="205" ht="36.2" customHeight="1" s="45"/>
-    <row r="206" ht="36.2" customHeight="1" s="45"/>
-    <row r="207" ht="33.95" customHeight="1" s="45"/>
-    <row r="208" ht="33.95" customHeight="1" s="45"/>
-    <row r="209" ht="33.95" customHeight="1" s="45"/>
-    <row r="210" ht="33.95" customHeight="1" s="45"/>
-    <row r="211" ht="33.95" customHeight="1" s="45"/>
-    <row r="212" ht="36.9" customHeight="1" s="45"/>
-    <row r="213" ht="36.9" customHeight="1" s="45"/>
-    <row r="214" ht="36.2" customHeight="1" s="45"/>
-    <row r="215" ht="36.2" customHeight="1" s="45"/>
-    <row r="216" ht="36.2" customHeight="1" s="45"/>
-    <row r="217" ht="36.2" customHeight="1" s="45"/>
-    <row r="218" ht="36.2" customHeight="1" s="45"/>
-    <row r="219" ht="33.95" customHeight="1" s="45"/>
-    <row r="220" ht="33.95" customHeight="1" s="45"/>
-    <row r="221" ht="33.95" customHeight="1" s="45"/>
-    <row r="222" ht="33.95" customHeight="1" s="45"/>
-    <row r="223" ht="36.9" customHeight="1" s="45"/>
-    <row r="224" ht="36.9" customHeight="1" s="45"/>
-    <row r="225" ht="33.95" customHeight="1" s="45"/>
-    <row r="226" ht="33.95" customHeight="1" s="45"/>
-    <row r="227" ht="33.95" customHeight="1" s="45"/>
-    <row r="228" ht="33.95" customHeight="1" s="45"/>
-    <row r="229" ht="36.9" customHeight="1" s="45"/>
-    <row r="230" ht="36.9" customHeight="1" s="45"/>
-    <row r="231" ht="36.2" customHeight="1" s="45"/>
-    <row r="232" ht="36.2" customHeight="1" s="45"/>
-    <row r="233" ht="33.95" customHeight="1" s="45"/>
-    <row r="234" ht="33.95" customHeight="1" s="45"/>
-    <row r="235" ht="33.95" customHeight="1" s="45"/>
-    <row r="236" ht="33.95" customHeight="1" s="45"/>
-    <row r="237" ht="36.9" customHeight="1" s="45"/>
-    <row r="238" ht="36.9" customHeight="1" s="45"/>
-    <row r="239" ht="36.9" customHeight="1" s="45"/>
-    <row r="240" ht="33.95" customHeight="1" s="45"/>
-    <row r="241" ht="33.95" customHeight="1" s="45"/>
-    <row r="242" ht="33.95" customHeight="1" s="45"/>
-    <row r="243" ht="36.9" customHeight="1" s="45"/>
-    <row r="244" ht="33.95" customHeight="1" s="45"/>
-    <row r="245" ht="33.95" customHeight="1" s="45"/>
-    <row r="246" ht="33.95" customHeight="1" s="45"/>
-    <row r="247" ht="33.95" customHeight="1" s="45"/>
-    <row r="248" ht="36.2" customHeight="1" s="45"/>
-    <row r="249" ht="36.2" customHeight="1" s="45"/>
-    <row r="250" ht="36.2" customHeight="1" s="45"/>
-    <row r="251" ht="36.2" customHeight="1" s="45"/>
-    <row r="252" ht="36.2" customHeight="1" s="45"/>
-    <row r="253" ht="36.9" customHeight="1" s="45"/>
-    <row r="254" ht="36.9" customHeight="1" s="45"/>
-    <row r="255" ht="33.95" customHeight="1" s="45"/>
-    <row r="256" ht="33.95" customHeight="1" s="45"/>
-    <row r="257" ht="33.95" customHeight="1" s="45"/>
-    <row r="258" ht="33.95" customHeight="1" s="45"/>
-    <row r="259" ht="33.95" customHeight="1" s="45"/>
-    <row r="260" ht="36.9" customHeight="1" s="45"/>
-    <row r="261" ht="36.9" customHeight="1" s="45"/>
-    <row r="262" ht="33.95" customHeight="1" s="45"/>
-    <row r="263" ht="33.95" customHeight="1" s="45"/>
-    <row r="264" ht="33.95" customHeight="1" s="45"/>
-    <row r="265" ht="33.95" customHeight="1" s="45"/>
-    <row r="266" ht="36.2" customHeight="1" s="45"/>
-    <row r="267" ht="36.2" customHeight="1" s="45"/>
-    <row r="268" ht="36.2" customHeight="1" s="45"/>
-    <row r="269" ht="36.2" customHeight="1" s="45"/>
-    <row r="270" ht="36.2" customHeight="1" s="45"/>
-    <row r="271" ht="36.9" customHeight="1" s="45"/>
-    <row r="272" ht="36.9" customHeight="1" s="45"/>
-    <row r="273" ht="33.95" customHeight="1" s="45"/>
-    <row r="274" ht="33.95" customHeight="1" s="45"/>
-    <row r="275" ht="33.95" customHeight="1" s="45"/>
-    <row r="276" ht="33.95" customHeight="1" s="45"/>
-    <row r="277" ht="33.95" customHeight="1" s="45"/>
-    <row r="278" ht="33.95" customHeight="1" s="45"/>
-    <row r="279" ht="33.95" customHeight="1" s="45"/>
-    <row r="280" ht="36.9" customHeight="1" s="45"/>
-    <row r="281" ht="36.9" customHeight="1" s="45"/>
-    <row r="282" ht="33.95" customHeight="1" s="45"/>
-    <row r="283" ht="33.95" customHeight="1" s="45"/>
-    <row r="284" ht="33.95" customHeight="1" s="45"/>
-    <row r="285" ht="36.9" customHeight="1" s="45"/>
-    <row r="286" ht="36.9" customHeight="1" s="45"/>
-    <row r="287" ht="36.9" customHeight="1" s="45"/>
-    <row r="288" ht="33.95" customHeight="1" s="45"/>
-    <row r="289" ht="33.95" customHeight="1" s="45"/>
-    <row r="290" ht="33.95" customHeight="1" s="45"/>
-    <row r="291" ht="33.95" customHeight="1" s="45"/>
-    <row r="292" ht="36.2" customHeight="1" s="45"/>
-    <row r="293" ht="36.2" customHeight="1" s="45"/>
-    <row r="294" ht="36.2" customHeight="1" s="45"/>
-    <row r="295" ht="36.2" customHeight="1" s="45"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2286,465 +3152,6 @@
       <c r="I2" s="42" t="n"/>
       <c r="J2" s="25" t="n"/>
     </row>
-    <row r="3" ht="34.45" customHeight="1" s="45"/>
-    <row r="4" ht="33.95" customHeight="1" s="45"/>
-    <row r="5" ht="36.9" customHeight="1" s="45"/>
-    <row r="6" ht="33.95" customHeight="1" s="45"/>
-    <row r="7" ht="33.95" customHeight="1" s="45"/>
-    <row r="8" ht="36.9" customHeight="1" s="45"/>
-    <row r="9" ht="36.9" customHeight="1" s="45"/>
-    <row r="10" ht="36.2" customHeight="1" s="45"/>
-    <row r="11" ht="36.2" customHeight="1" s="45"/>
-    <row r="12" ht="36.9" customHeight="1" s="45"/>
-    <row r="13" ht="36.9" customHeight="1" s="45"/>
-    <row r="14" ht="34.4" customHeight="1" s="45"/>
-    <row r="15" ht="34.4" customHeight="1" s="45"/>
-    <row r="16" ht="34.4" customHeight="1" s="45"/>
-    <row r="17" ht="36.2" customHeight="1" s="45"/>
-    <row r="18" ht="36.2" customHeight="1" s="45"/>
-    <row r="19" ht="36.2" customHeight="1" s="45"/>
-    <row r="20" ht="36.2" customHeight="1" s="45"/>
-    <row r="21" ht="36.9" customHeight="1" s="45"/>
-    <row r="22" ht="36.9" customHeight="1" s="45"/>
-    <row r="23" ht="36.9" customHeight="1" s="45"/>
-    <row r="24" ht="36.9" customHeight="1" s="45"/>
-    <row r="25" ht="34.4" customHeight="1" s="45"/>
-    <row r="26" ht="34.4" customHeight="1" s="45"/>
-    <row r="27" ht="34.4" customHeight="1" s="45"/>
-    <row r="28" ht="33.95" customHeight="1" s="45"/>
-    <row r="29" ht="33.95" customHeight="1" s="45"/>
-    <row r="30" ht="33.95" customHeight="1" s="45"/>
-    <row r="31" ht="36.2" customHeight="1" s="45"/>
-    <row r="32" ht="36.2" customHeight="1" s="45"/>
-    <row r="33" ht="36.2" customHeight="1" s="45"/>
-    <row r="34" ht="36.2" customHeight="1" s="45"/>
-    <row r="35" ht="36.2" customHeight="1" s="45"/>
-    <row r="36" ht="36.2" customHeight="1" s="45"/>
-    <row r="37" ht="36.2" customHeight="1" s="45"/>
-    <row r="38" ht="36.2" customHeight="1" s="45"/>
-    <row r="39" ht="34.4" customHeight="1" s="45"/>
-    <row r="40" ht="34.4" customHeight="1" s="45"/>
-    <row r="41" ht="34.4" customHeight="1" s="45"/>
-    <row r="42" ht="34.4" customHeight="1" s="45"/>
-    <row r="43" ht="36.2" customHeight="1" s="45"/>
-    <row r="44" ht="36.2" customHeight="1" s="45"/>
-    <row r="45" ht="36.9" customHeight="1" s="45"/>
-    <row r="46" ht="36.9" customHeight="1" s="45"/>
-    <row r="47" ht="34.4" customHeight="1" s="45"/>
-    <row r="48" ht="36.9" customHeight="1" s="45"/>
-    <row r="49" ht="34.4" customHeight="1" s="45"/>
-    <row r="50" ht="34.4" customHeight="1" s="45"/>
-    <row r="51" ht="36.9" customHeight="1" s="45"/>
-    <row r="52" ht="36.2" customHeight="1" s="45"/>
-    <row r="53" ht="36.2" customHeight="1" s="45"/>
-    <row r="54" ht="36.2" customHeight="1" s="45"/>
-    <row r="55" ht="34.4" customHeight="1" s="45"/>
-    <row r="56" ht="34.4" customHeight="1" s="45"/>
-    <row r="57" ht="34.4" customHeight="1" s="45"/>
-    <row r="58" ht="36.9" customHeight="1" s="45"/>
-    <row r="59" ht="36.9" customHeight="1" s="45"/>
-    <row r="60" ht="36.2" customHeight="1" s="45"/>
-    <row r="61" ht="36.2" customHeight="1" s="45"/>
-    <row r="62" ht="34.4" customHeight="1" s="45"/>
-    <row r="63" ht="34.4" customHeight="1" s="45"/>
-    <row r="64" ht="34.4" customHeight="1" s="45"/>
-    <row r="65" ht="34.4" customHeight="1" s="45"/>
-    <row r="66" ht="36.9" customHeight="1" s="45"/>
-    <row r="67" ht="34.4" customHeight="1" s="45"/>
-    <row r="68" ht="36.9" customHeight="1" s="45"/>
-    <row r="69" ht="34.4" customHeight="1" s="45"/>
-    <row r="70" ht="36.9" customHeight="1" s="45"/>
-    <row r="71" ht="34.4" customHeight="1" s="45"/>
-    <row r="72" ht="34.4" customHeight="1" s="45"/>
-    <row r="73" ht="34.4" customHeight="1" s="45"/>
-    <row r="74" ht="36.9" customHeight="1" s="45"/>
-    <row r="75" ht="36.9" customHeight="1" s="45"/>
-    <row r="76" ht="34.4" customHeight="1" s="45"/>
-    <row r="77" ht="34.4" customHeight="1" s="45"/>
-    <row r="78" ht="34.4" customHeight="1" s="45"/>
-    <row r="79" ht="36.9" customHeight="1" s="45"/>
-    <row r="80" ht="36.9" customHeight="1" s="45"/>
-    <row r="81" ht="36.9" customHeight="1" s="45"/>
-    <row r="82" ht="33.95" customHeight="1" s="45"/>
-    <row r="83" ht="33.95" customHeight="1" s="45"/>
-    <row r="84" ht="33.95" customHeight="1" s="45"/>
-    <row r="85" ht="33.95" customHeight="1" s="45"/>
-    <row r="86" ht="36.2" customHeight="1" s="45"/>
-    <row r="87" ht="36.2" customHeight="1" s="45"/>
-    <row r="88" ht="36.2" customHeight="1" s="45"/>
-    <row r="89" ht="36.2" customHeight="1" s="45"/>
-    <row r="90" ht="36.2" customHeight="1" s="45"/>
-    <row r="91" ht="36.2" customHeight="1" s="45"/>
-    <row r="92" ht="36.2" customHeight="1" s="45"/>
-    <row r="93" ht="36.2" customHeight="1" s="45"/>
-    <row r="94" ht="36.2" customHeight="1" s="45"/>
-    <row r="95" ht="36.2" customHeight="1" s="45"/>
-    <row r="96" ht="36.2" customHeight="1" s="45"/>
-    <row r="97" ht="36.9" customHeight="1" s="45"/>
-    <row r="98" ht="36.9" customHeight="1" s="45"/>
-    <row r="99" ht="33.95" customHeight="1" s="45"/>
-    <row r="100" ht="33.95" customHeight="1" s="45"/>
-    <row r="101" ht="33.95" customHeight="1" s="45"/>
-    <row r="102" ht="36.9" customHeight="1" s="45"/>
-    <row r="103" ht="33.95" customHeight="1" s="45"/>
-    <row r="104" ht="33.95" customHeight="1" s="45"/>
-    <row r="105" ht="33.95" customHeight="1" s="45"/>
-    <row r="106" ht="33.95" customHeight="1" s="45"/>
-    <row r="107" ht="36.2" customHeight="1" s="45"/>
-    <row r="108" ht="36.2" customHeight="1" s="45"/>
-    <row r="109" ht="36.2" customHeight="1" s="45"/>
-    <row r="110" ht="36.2" customHeight="1" s="45"/>
-    <row r="111" ht="33.95" customHeight="1" s="45"/>
-    <row r="112" ht="33.95" customHeight="1" s="45"/>
-    <row r="113" ht="33.95" customHeight="1" s="45"/>
-    <row r="114" ht="36.9" customHeight="1" s="45"/>
-    <row r="115" ht="36.9" customHeight="1" s="45"/>
-    <row r="116" ht="36.2" customHeight="1" s="45"/>
-    <row r="117" ht="36.2" customHeight="1" s="45"/>
-    <row r="118" ht="33.95" customHeight="1" s="45"/>
-    <row r="119" ht="33.95" customHeight="1" s="45"/>
-    <row r="120" ht="33.95" customHeight="1" s="45"/>
-    <row r="121" ht="33.95" customHeight="1" s="45"/>
-    <row r="122" ht="36.9" customHeight="1" s="45"/>
-    <row r="123" ht="36.9" customHeight="1" s="45"/>
-    <row r="124" ht="36.2" customHeight="1" s="45"/>
-    <row r="125" ht="36.2" customHeight="1" s="45"/>
-    <row r="126" ht="33.95" customHeight="1" s="45"/>
-    <row r="127" ht="33.95" customHeight="1" s="45"/>
-    <row r="128" ht="33.95" customHeight="1" s="45"/>
-    <row r="129" ht="33.95" customHeight="1" s="45"/>
-    <row r="130" ht="36.9" customHeight="1" s="45"/>
-    <row r="131" ht="36.9" customHeight="1" s="45"/>
-    <row r="132" ht="36.2" customHeight="1" s="45"/>
-    <row r="133" ht="36.2" customHeight="1" s="45"/>
-    <row r="134" ht="33.95" customHeight="1" s="45"/>
-    <row r="135" ht="33.95" customHeight="1" s="45"/>
-    <row r="136" ht="33.95" customHeight="1" s="45"/>
-    <row r="137" ht="36.9" customHeight="1" s="45"/>
-    <row r="138" ht="36.9" customHeight="1" s="45"/>
-    <row r="139" ht="33.95" customHeight="1" s="45"/>
-    <row r="140" ht="33.95" customHeight="1" s="45"/>
-    <row r="141" ht="33.95" customHeight="1" s="45"/>
-    <row r="142" ht="33.95" customHeight="1" s="45"/>
-    <row r="143" ht="36.2" customHeight="1" s="45"/>
-    <row r="144" ht="36.2" customHeight="1" s="45"/>
-    <row r="145" ht="36.2" customHeight="1" s="45"/>
-    <row r="146" ht="33.95" customHeight="1" s="45"/>
-    <row r="147" ht="33.95" customHeight="1" s="45"/>
-    <row r="148" ht="33.95" customHeight="1" s="45"/>
-    <row r="149" ht="36.9" customHeight="1" s="45"/>
-    <row r="150" ht="36.9" customHeight="1" s="45"/>
-    <row r="151" ht="36.9" customHeight="1" s="45"/>
-    <row r="152" ht="36.9" customHeight="1" s="45"/>
-    <row r="153" ht="33.95" customHeight="1" s="45"/>
-    <row r="154" ht="33.95" customHeight="1" s="45"/>
-    <row r="155" ht="33.95" customHeight="1" s="45"/>
-    <row r="156" ht="33.95" customHeight="1" s="45"/>
-    <row r="157" ht="33.95" customHeight="1" s="45"/>
-    <row r="158" ht="33.95" customHeight="1" s="45"/>
-    <row r="159" ht="33.95" customHeight="1" s="45"/>
-    <row r="160" ht="33.95" customHeight="1" s="45"/>
-    <row r="161" ht="36.9" customHeight="1" s="45"/>
-    <row r="162" ht="36.9" customHeight="1" s="45"/>
-    <row r="163" ht="33.95" customHeight="1" s="45"/>
-    <row r="164" ht="33.95" customHeight="1" s="45"/>
-    <row r="165" ht="33.95" customHeight="1" s="45"/>
-    <row r="166" ht="36.9" customHeight="1" s="45"/>
-    <row r="167" ht="36.9" customHeight="1" s="45"/>
-    <row r="168" ht="36.9" customHeight="1" s="45"/>
-    <row r="169" ht="36.9" customHeight="1" s="45"/>
-    <row r="170" ht="33.95" customHeight="1" s="45"/>
-    <row r="171" ht="33.95" customHeight="1" s="45"/>
-    <row r="172" ht="36.9" customHeight="1" s="45"/>
-    <row r="173" ht="33.95" customHeight="1" s="45"/>
-    <row r="174" ht="33.95" customHeight="1" s="45"/>
-    <row r="175" ht="33.95" customHeight="1" s="45"/>
-    <row r="176" ht="36.2" customHeight="1" s="45"/>
-    <row r="177" ht="36.2" customHeight="1" s="45"/>
-    <row r="178" ht="36.2" customHeight="1" s="45"/>
-    <row r="179" ht="36.2" customHeight="1" s="45"/>
-    <row r="180" ht="33.95" customHeight="1" s="45"/>
-    <row r="181" ht="33.95" customHeight="1" s="45"/>
-    <row r="182" ht="33.95" customHeight="1" s="45"/>
-    <row r="183" ht="36.9" customHeight="1" s="45"/>
-    <row r="184" ht="36.9" customHeight="1" s="45"/>
-    <row r="185" ht="36.2" customHeight="1" s="45"/>
-    <row r="186" ht="36.2" customHeight="1" s="45"/>
-    <row r="187" ht="36.2" customHeight="1" s="45"/>
-    <row r="188" ht="36.2" customHeight="1" s="45"/>
-    <row r="189" ht="33.95" customHeight="1" s="45"/>
-    <row r="190" ht="33.95" customHeight="1" s="45"/>
-    <row r="191" ht="33.95" customHeight="1" s="45"/>
-    <row r="192" ht="36.9" customHeight="1" s="45"/>
-    <row r="193" ht="36.9" customHeight="1" s="45"/>
-    <row r="194" ht="33.95" customHeight="1" s="45"/>
-    <row r="195" ht="33.95" customHeight="1" s="45"/>
-    <row r="196" ht="33.95" customHeight="1" s="45"/>
-    <row r="197" ht="33.95" customHeight="1" s="45"/>
-    <row r="198" ht="36.9" customHeight="1" s="45"/>
-    <row r="199" ht="36.9" customHeight="1" s="45"/>
-    <row r="200" ht="33.95" customHeight="1" s="45"/>
-    <row r="201" ht="33.95" customHeight="1" s="45"/>
-    <row r="202" ht="33.95" customHeight="1" s="45"/>
-    <row r="203" ht="33.95" customHeight="1" s="45"/>
-    <row r="204" ht="36.2" customHeight="1" s="45"/>
-    <row r="205" ht="36.2" customHeight="1" s="45"/>
-    <row r="206" ht="36.2" customHeight="1" s="45"/>
-    <row r="207" ht="33.95" customHeight="1" s="45"/>
-    <row r="208" ht="33.95" customHeight="1" s="45"/>
-    <row r="209" ht="33.95" customHeight="1" s="45"/>
-    <row r="210" ht="33.95" customHeight="1" s="45"/>
-    <row r="211" ht="33.95" customHeight="1" s="45"/>
-    <row r="212" ht="36.9" customHeight="1" s="45"/>
-    <row r="213" ht="36.9" customHeight="1" s="45"/>
-    <row r="214" ht="36.2" customHeight="1" s="45"/>
-    <row r="215" ht="36.2" customHeight="1" s="45"/>
-    <row r="216" ht="36.2" customHeight="1" s="45"/>
-    <row r="217" ht="36.2" customHeight="1" s="45"/>
-    <row r="218" ht="36.2" customHeight="1" s="45"/>
-    <row r="219" ht="33.95" customHeight="1" s="45"/>
-    <row r="220" ht="33.95" customHeight="1" s="45"/>
-    <row r="221" ht="33.95" customHeight="1" s="45"/>
-    <row r="222" ht="33.95" customHeight="1" s="45"/>
-    <row r="223" ht="36.9" customHeight="1" s="45"/>
-    <row r="224" ht="36.9" customHeight="1" s="45"/>
-    <row r="225" ht="33.95" customHeight="1" s="45"/>
-    <row r="226" ht="33.95" customHeight="1" s="45"/>
-    <row r="227" ht="33.95" customHeight="1" s="45"/>
-    <row r="228" ht="33.95" customHeight="1" s="45"/>
-    <row r="229" ht="36.9" customHeight="1" s="45"/>
-    <row r="230" ht="36.9" customHeight="1" s="45"/>
-    <row r="231" ht="36.2" customHeight="1" s="45"/>
-    <row r="232" ht="36.2" customHeight="1" s="45"/>
-    <row r="233" ht="33.95" customHeight="1" s="45"/>
-    <row r="234" ht="33.95" customHeight="1" s="45"/>
-    <row r="235" ht="33.95" customHeight="1" s="45"/>
-    <row r="236" ht="33.95" customHeight="1" s="45"/>
-    <row r="237" ht="36.9" customHeight="1" s="45"/>
-    <row r="238" ht="36.9" customHeight="1" s="45"/>
-    <row r="239" ht="36.9" customHeight="1" s="45"/>
-    <row r="240" ht="33.95" customHeight="1" s="45"/>
-    <row r="241" ht="33.95" customHeight="1" s="45"/>
-    <row r="242" ht="33.95" customHeight="1" s="45"/>
-    <row r="243" ht="36.9" customHeight="1" s="45"/>
-    <row r="244" ht="33.95" customHeight="1" s="45"/>
-    <row r="245" ht="33.95" customHeight="1" s="45"/>
-    <row r="246" ht="33.95" customHeight="1" s="45"/>
-    <row r="247" ht="33.95" customHeight="1" s="45"/>
-    <row r="248" ht="36.2" customHeight="1" s="45"/>
-    <row r="249" ht="36.2" customHeight="1" s="45"/>
-    <row r="250" ht="36.2" customHeight="1" s="45"/>
-    <row r="251" ht="36.2" customHeight="1" s="45"/>
-    <row r="252" ht="36.2" customHeight="1" s="45"/>
-    <row r="253" ht="36.9" customHeight="1" s="45"/>
-    <row r="254" ht="36.9" customHeight="1" s="45"/>
-    <row r="255" ht="33.95" customHeight="1" s="45"/>
-    <row r="256" ht="33.95" customHeight="1" s="45"/>
-    <row r="257" ht="33.95" customHeight="1" s="45"/>
-    <row r="258" ht="33.95" customHeight="1" s="45"/>
-    <row r="259" ht="33.95" customHeight="1" s="45"/>
-    <row r="260" ht="36.9" customHeight="1" s="45"/>
-    <row r="261" ht="36.9" customHeight="1" s="45"/>
-    <row r="262" ht="33.95" customHeight="1" s="45"/>
-    <row r="263" ht="33.95" customHeight="1" s="45"/>
-    <row r="264" ht="33.95" customHeight="1" s="45"/>
-    <row r="265" ht="33.95" customHeight="1" s="45"/>
-    <row r="266" ht="36.2" customHeight="1" s="45"/>
-    <row r="267" ht="36.2" customHeight="1" s="45"/>
-    <row r="268" ht="36.2" customHeight="1" s="45"/>
-    <row r="269" ht="36.2" customHeight="1" s="45"/>
-    <row r="270" ht="36.2" customHeight="1" s="45"/>
-    <row r="271" ht="36.9" customHeight="1" s="45"/>
-    <row r="272" ht="36.9" customHeight="1" s="45"/>
-    <row r="273" ht="33.95" customHeight="1" s="45"/>
-    <row r="274" ht="33.95" customHeight="1" s="45"/>
-    <row r="275" ht="33.95" customHeight="1" s="45"/>
-    <row r="276" ht="33.95" customHeight="1" s="45"/>
-    <row r="277" ht="33.95" customHeight="1" s="45"/>
-    <row r="278" ht="33.95" customHeight="1" s="45"/>
-    <row r="279" ht="33.95" customHeight="1" s="45"/>
-    <row r="280" ht="36.9" customHeight="1" s="45"/>
-    <row r="281" ht="36.9" customHeight="1" s="45"/>
-    <row r="282" ht="33.95" customHeight="1" s="45"/>
-    <row r="283" ht="33.95" customHeight="1" s="45"/>
-    <row r="284" ht="33.95" customHeight="1" s="45"/>
-    <row r="285" ht="36.9" customHeight="1" s="45"/>
-    <row r="286" ht="36.9" customHeight="1" s="45"/>
-    <row r="287" ht="36.9" customHeight="1" s="45"/>
-    <row r="288" ht="33.95" customHeight="1" s="45"/>
-    <row r="289" ht="33.95" customHeight="1" s="45"/>
-    <row r="290" ht="33.95" customHeight="1" s="45"/>
-    <row r="291" ht="33.95" customHeight="1" s="45"/>
-    <row r="292" ht="36.2" customHeight="1" s="45"/>
-    <row r="293" ht="36.2" customHeight="1" s="45"/>
-    <row r="294" ht="36.2" customHeight="1" s="45"/>
-    <row r="295" ht="36.2" customHeight="1" s="45"/>
-    <row r="300" ht="36.9" customHeight="1" s="45"/>
-    <row r="301" ht="36.9" customHeight="1" s="45"/>
-    <row r="302" ht="33.95" customHeight="1" s="45"/>
-    <row r="303" ht="33.95" customHeight="1" s="45"/>
-    <row r="304" ht="33.95" customHeight="1" s="45"/>
-    <row r="305" ht="33.95" customHeight="1" s="45"/>
-    <row r="306" ht="33.95" customHeight="1" s="45"/>
-    <row r="307" ht="36.2" customHeight="1" s="45"/>
-    <row r="308" ht="36.2" customHeight="1" s="45"/>
-    <row r="309" ht="36.9" customHeight="1" s="45"/>
-    <row r="310" ht="36.9" customHeight="1" s="45"/>
-    <row r="311" ht="33.95" customHeight="1" s="45"/>
-    <row r="312" ht="33.95" customHeight="1" s="45"/>
-    <row r="313" ht="33.95" customHeight="1" s="45"/>
-    <row r="314" ht="33.95" customHeight="1" s="45"/>
-    <row r="315" ht="36.2" customHeight="1" s="45"/>
-    <row r="316" ht="36.2" customHeight="1" s="45"/>
-    <row r="317" ht="33.95" customHeight="1" s="45"/>
-    <row r="318" ht="81.8" customHeight="1" s="45"/>
-    <row r="319" ht="77.75" customHeight="1" s="45"/>
-    <row r="320" ht="62.15" customHeight="1" s="45"/>
-    <row r="321" ht="33.95" customHeight="1" s="45"/>
-    <row r="322" ht="33.95" customHeight="1" s="45"/>
-    <row r="323" ht="33.95" customHeight="1" s="45"/>
-    <row r="324" ht="33.95" customHeight="1" s="45"/>
-    <row r="325" ht="36.9" customHeight="1" s="45"/>
-    <row r="326" ht="36.9" customHeight="1" s="45"/>
-    <row r="327" ht="36.2" customHeight="1" s="45"/>
-    <row r="328" ht="36.2" customHeight="1" s="45"/>
-    <row r="329" ht="36.2" customHeight="1" s="45"/>
-    <row r="330" ht="75" customHeight="1" s="45"/>
-    <row r="331" ht="75" customHeight="1" s="45"/>
-    <row r="332" ht="36.9" customHeight="1" s="45"/>
-    <row r="333" ht="36.9" customHeight="1" s="45"/>
-    <row r="334" ht="33.95" customHeight="1" s="45"/>
-    <row r="335" ht="33.95" customHeight="1" s="45"/>
-    <row r="336" ht="33.95" customHeight="1" s="45"/>
-    <row r="337" ht="33.95" customHeight="1" s="45"/>
-    <row r="338" ht="33.95" customHeight="1" s="45"/>
-    <row r="339" ht="33.95" customHeight="1" s="45"/>
-    <row r="340" ht="33.95" customHeight="1" s="45"/>
-    <row r="341" ht="36.9" customHeight="1" s="45"/>
-    <row r="342" ht="36.9" customHeight="1" s="45"/>
-    <row r="343" ht="36.2" customHeight="1" s="45"/>
-    <row r="344" ht="36.2" customHeight="1" s="45"/>
-    <row r="345" ht="75" customHeight="1" s="45"/>
-    <row r="346" ht="75" customHeight="1" s="45"/>
-    <row r="347" ht="36.9" customHeight="1" s="45"/>
-    <row r="348" ht="36.9" customHeight="1" s="45"/>
-    <row r="349" ht="33.95" customHeight="1" s="45"/>
-    <row r="350" ht="33.95" customHeight="1" s="45"/>
-    <row r="351" ht="33.95" customHeight="1" s="45"/>
-    <row r="352" ht="36.9" customHeight="1" s="45"/>
-    <row r="353" ht="36.9" customHeight="1" s="45"/>
-    <row r="354" ht="36.9" customHeight="1" s="45"/>
-    <row r="355" ht="36.9" customHeight="1" s="45"/>
-    <row r="356" ht="33.95" customHeight="1" s="45"/>
-    <row r="357" ht="33.95" customHeight="1" s="45"/>
-    <row r="358" ht="33.95" customHeight="1" s="45"/>
-    <row r="359" ht="33.95" customHeight="1" s="45"/>
-    <row r="360" ht="33.95" customHeight="1" s="45"/>
-    <row r="361" ht="33.95" customHeight="1" s="45"/>
-    <row r="362" ht="33.95" customHeight="1" s="45"/>
-    <row r="363" ht="36.9" customHeight="1" s="45"/>
-    <row r="364" ht="36.9" customHeight="1" s="45"/>
-    <row r="365" ht="36.2" customHeight="1" s="45"/>
-    <row r="366" ht="36.2" customHeight="1" s="45"/>
-    <row r="367" ht="36.2" customHeight="1" s="45"/>
-    <row r="368" ht="36.2" customHeight="1" s="45"/>
-    <row r="369" ht="36.2" customHeight="1" s="45"/>
-    <row r="370" ht="36.9" customHeight="1" s="45"/>
-    <row r="371" ht="36.9" customHeight="1" s="45"/>
-    <row r="372" ht="33.95" customHeight="1" s="45"/>
-    <row r="373" ht="33.95" customHeight="1" s="45"/>
-    <row r="374" ht="33.95" customHeight="1" s="45"/>
-    <row r="375" ht="33.95" customHeight="1" s="45"/>
-    <row r="376" ht="33.95" customHeight="1" s="45"/>
-    <row r="377" ht="33.95" customHeight="1" s="45"/>
-    <row r="378" ht="33.95" customHeight="1" s="45"/>
-    <row r="379" ht="33.95" customHeight="1" s="45"/>
-    <row r="380" ht="36.9" customHeight="1" s="45"/>
-    <row r="381" ht="36.9" customHeight="1" s="45"/>
-    <row r="382" ht="33.95" customHeight="1" s="45"/>
-    <row r="383" ht="33.95" customHeight="1" s="45"/>
-    <row r="384" ht="33.95" customHeight="1" s="45"/>
-    <row r="385" ht="36.9" customHeight="1" s="45"/>
-    <row r="386" ht="36.9" customHeight="1" s="45"/>
-    <row r="387" ht="36.2" customHeight="1" s="45"/>
-    <row r="388" ht="36.2" customHeight="1" s="45"/>
-    <row r="389" ht="36.2" customHeight="1" s="45"/>
-    <row r="390" ht="36.2" customHeight="1" s="45"/>
-    <row r="391" ht="33.95" customHeight="1" s="45"/>
-    <row r="392" ht="33.95" customHeight="1" s="45"/>
-    <row r="393" ht="36.9" customHeight="1" s="45"/>
-    <row r="394" ht="36.9" customHeight="1" s="45"/>
-    <row r="395" ht="36.9" customHeight="1" s="45"/>
-    <row r="396" ht="33.95" customHeight="1" s="45"/>
-    <row r="397" ht="33.95" customHeight="1" s="45"/>
-    <row r="398" ht="33.95" customHeight="1" s="45"/>
-    <row r="399" ht="33.95" customHeight="1" s="45"/>
-    <row r="400" ht="36.9" customHeight="1" s="45"/>
-    <row r="401" ht="36.9" customHeight="1" s="45"/>
-    <row r="402" ht="36.9" customHeight="1" s="45"/>
-    <row r="403" ht="33.95" customHeight="1" s="45"/>
-    <row r="404" ht="33.95" customHeight="1" s="45"/>
-    <row r="405" ht="33.95" customHeight="1" s="45"/>
-    <row r="406" ht="33.95" customHeight="1" s="45"/>
-    <row r="407" ht="36.9" customHeight="1" s="45"/>
-    <row r="408" ht="36.9" customHeight="1" s="45"/>
-    <row r="409" ht="33.95" customHeight="1" s="45"/>
-    <row r="410" ht="33.95" customHeight="1" s="45"/>
-    <row r="411" ht="33.95" customHeight="1" s="45"/>
-    <row r="412" ht="33.95" customHeight="1" s="45"/>
-    <row r="413" ht="33.95" customHeight="1" s="45"/>
-    <row r="414" ht="36.9" customHeight="1" s="45"/>
-    <row r="415" ht="36.9" customHeight="1" s="45"/>
-    <row r="416" ht="36.2" customHeight="1" s="45"/>
-    <row r="417" ht="36.2" customHeight="1" s="45"/>
-    <row r="418" ht="36.2" customHeight="1" s="45"/>
-    <row r="419" ht="36.2" customHeight="1" s="45"/>
-    <row r="420" ht="36.2" customHeight="1" s="45"/>
-    <row r="421" ht="36.9" customHeight="1" s="45"/>
-    <row r="422" ht="36.9" customHeight="1" s="45"/>
-    <row r="423" ht="33.95" customHeight="1" s="45"/>
-    <row r="424" ht="33.95" customHeight="1" s="45"/>
-    <row r="425" ht="33.95" customHeight="1" s="45"/>
-    <row r="426" ht="33.95" customHeight="1" s="45"/>
-    <row r="427" ht="33.95" customHeight="1" s="45"/>
-    <row r="428" ht="33.95" customHeight="1" s="45"/>
-    <row r="429" ht="36.9" customHeight="1" s="45"/>
-    <row r="430" ht="36.9" customHeight="1" s="45"/>
-    <row r="431" ht="36.2" customHeight="1" s="45"/>
-    <row r="432" ht="36.2" customHeight="1" s="45"/>
-    <row r="433" ht="36.2" customHeight="1" s="45"/>
-    <row r="434" ht="33.95" customHeight="1" s="45"/>
-    <row r="435" ht="33.95" customHeight="1" s="45"/>
-    <row r="436" ht="36.9" customHeight="1" s="45"/>
-    <row r="437" ht="36.9" customHeight="1" s="45"/>
-    <row r="438" ht="36.9" customHeight="1" s="45"/>
-    <row r="439" ht="36.9" customHeight="1" s="45"/>
-    <row r="440" ht="33.95" customHeight="1" s="45"/>
-    <row r="441" ht="33.95" customHeight="1" s="45"/>
-    <row r="442" ht="33.95" customHeight="1" s="45"/>
-    <row r="443" ht="36.2" customHeight="1" s="45"/>
-    <row r="444" ht="36.2" customHeight="1" s="45"/>
-    <row r="445" ht="36.2" customHeight="1" s="45"/>
-    <row r="446" ht="33.95" customHeight="1" s="45"/>
-    <row r="447" ht="33.95" customHeight="1" s="45"/>
-    <row r="448" ht="36.9" customHeight="1" s="45"/>
-    <row r="449" ht="36.9" customHeight="1" s="45"/>
-    <row r="450" ht="36.9" customHeight="1" s="45"/>
-    <row r="451" ht="36.9" customHeight="1" s="45"/>
-    <row r="452" ht="33.95" customHeight="1" s="45"/>
-    <row r="453" ht="33.95" customHeight="1" s="45"/>
-    <row r="454" ht="33.95" customHeight="1" s="45"/>
-    <row r="455" ht="33.95" customHeight="1" s="45"/>
-    <row r="456" ht="36.9" customHeight="1" s="45"/>
-    <row r="457" ht="36.9" customHeight="1" s="45"/>
-    <row r="458" ht="33.95" customHeight="1" s="45"/>
-    <row r="459" ht="33.95" customHeight="1" s="45"/>
-    <row r="460" ht="36.9" customHeight="1" s="45"/>
-    <row r="461" ht="36.9" customHeight="1" s="45"/>
-    <row r="462" ht="36.9" customHeight="1" s="45"/>
-    <row r="463" ht="33.95" customHeight="1" s="45"/>
-    <row r="464" ht="33.95" customHeight="1" s="45"/>
-    <row r="465" ht="33.95" customHeight="1" s="45"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2769,8 +3176,8 @@
     <col width="15.8888888888889" customWidth="1" style="23" min="9" max="9"/>
     <col width="30" customWidth="1" style="23" min="10" max="10"/>
     <col width="11.7777777777778" customWidth="1" style="25" min="11" max="11"/>
-    <col width="18" customWidth="1" style="25" min="12" max="12"/>
-    <col width="18" customWidth="1" style="25" min="13" max="13"/>
+    <col width="12" customWidth="1" style="25" min="12" max="12"/>
+    <col width="16.8888888888889" customWidth="1" style="25" min="13" max="13"/>
     <col width="11.3333333333333" customWidth="1" style="25" min="14" max="16384"/>
   </cols>
   <sheetData>
@@ -2794,24 +3201,25 @@
         <f>WEEKNUM(B1,2)</f>
         <v/>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="46" t="inlineStr">
         <is>
           <t>开始日期（含）</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="46" t="inlineStr">
         <is>
           <t>结束日期（含）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1" s="45">
-      <c r="A2" s="10" t="n">
-        <v>1</v>
+      <c r="A2" s="10">
+        <f>IF(AND(YEAR(L2)=YEAR(M2),MONTH(L2)=MONTH(M2)),MONTH(L2),"区间")</f>
+        <v/>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>区间出货抽检不良统计表</t>
+          <t>月出货抽检不良统计表</t>
         </is>
       </c>
       <c r="E2" s="12">
@@ -2833,10 +3241,10 @@
         </is>
       </c>
       <c r="J2" s="21" t="n"/>
-      <c r="L2" s="46" t="n">
+      <c r="L2" s="47" t="n">
         <v>46023</v>
       </c>
-      <c r="M2" s="46" t="n">
+      <c r="M2" s="47" t="n">
         <v>46053</v>
       </c>
     </row>
@@ -3205,10 +3613,7 @@
       <c r="H17" s="29" t="n"/>
       <c r="I17" s="23" t="n"/>
       <c r="J17" s="25" t="n"/>
-      <c r="M17" s="25">
-        <f>22/133</f>
-        <v/>
-      </c>
+      <c r="M17" s="25" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -3412,20 +3817,21 @@
       </c>
     </row>
     <row r="31">
-      <c r="L31" t="inlineStr">
+      <c r="L31" s="46" t="inlineStr">
         <is>
           <t>周开始（含）</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M31" s="46" t="inlineStr">
         <is>
           <t>周结束（含）</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22.5" customHeight="1" s="45">
-      <c r="A32" s="10" t="n">
-        <v>5</v>
+      <c r="A32" s="10">
+        <f>WEEKNUM(L32,21)</f>
+        <v/>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
@@ -3451,10 +3857,10 @@
         </is>
       </c>
       <c r="J32" s="21" t="n"/>
-      <c r="L32" s="46" t="n">
+      <c r="L32" s="47" t="n">
         <v>46048</v>
       </c>
-      <c r="M32" s="46" t="n">
+      <c r="M32" s="47" t="n">
         <v>46054</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: exclude rank values from original-form quantity charts
Release v1.1.1 with corrected bundled and external templates while preserving v1.1.0 UI improvements. Verified 57 tests, Ruff, and application smoke test.
</commit_message>
<xml_diff>
--- a/templates/成品日检表模板.xlsx
+++ b/templates/成品日检表模板.xlsx
@@ -2093,70 +2093,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <dLbls>
-            <numFmt formatCode="General"/>
-            <spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-            <txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr lang="zh-CN" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </txPr>
-            <dLblPos val="outEnd"/>
-            <showLegendKey val="0"/>
-            <showVal val="1"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showBubbleSize val="0"/>
-            <showLeaderLines val="0"/>
-          </dLbls>
-          <cat>
-            <strRef>
-              <f>数据分析表!$A$34:$A$57</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>数据分析表!$C$34:$C$57</f>
-            </numRef>
-          </val>
-        </ser>
         <dLbls>
           <showLegendKey val="0"/>
           <showVal val="1"/>

</xml_diff>